<commit_message>
feat: implement static web-based category sync auditor and auxiliary utility scripts
</commit_message>
<xml_diff>
--- a/test_audit/excel_margin_conflict.xlsx
+++ b/test_audit/excel_margin_conflict.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D4"/>
+  <dimension ref="A1:D5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -487,6 +487,24 @@
         <v>50</v>
       </c>
       <c r="D4" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>AVNBRA-EXP4</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>100</v>
+      </c>
+      <c r="C5" t="n">
+        <v>50</v>
+      </c>
+      <c r="D5" t="inlineStr">
         <is>
           <t>SIM</t>
         </is>

</xml_diff>